<commit_message>
PX-01: referencias virales por vídeo en la hoja de solicitudes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
@@ -781,10 +781,9 @@
       </c>
       <c r="D7" s="44" t="inlineStr">
         <is>
-          <t>FAA, Lessons Learned JA8119: https://www.faa.gov/lessons_learned/transport_airplane/accidents/JA8119
-Aviation Safety Network: https://aviation-safety.net/asndb/327151
-JAL Safety Promotion Center: https://www.jal.com/en-jp/safety/center/
-Estilo del canal (vídeo propio): https://youtu.be/v3ff8dfP-bs</t>
+          <t>«WHAT caused the WORST single air crash in history?? | Japan Air 123» — Green Dot Aviation — 3,9 M vistas — https://youtu.be/h3AWPhslRg4
+«Inside the Unprecedented Event on Japan Airlines Flight 123 | Mayday: Air Disaster» — Mayday: Air Disaster — 3,6 M vistas — https://youtu.be/ikh51ls7x0M
+«Inside The Deadliest Single-Aircraft Disaster Ever | Last Moments» — Qxir — 4,0 M vistas — https://youtu.be/1j71TkVv2q8</t>
         </is>
       </c>
       <c r="E7" s="44" t="inlineStr">
@@ -819,9 +818,9 @@
       </c>
       <c r="D8" s="48" t="inlineStr">
         <is>
-          <t>Informe final CIAIAC (PDF): https://www.transportes.gob.es/recursos_mfom/2008_032_a_eng_3.pdf
-Copia del informe en la FAA: https://www.faa.gov/sites/faa.gov/files/2022-11/Final%20CIAIAC%20Rpt%20Spanair%205022.pdf
-Asociación de afectados JK5022: https://avjk5022.com/vuelojk5022</t>
+          <t>«The flight that CRASHED after 10 seconds | Spanair 5022» — Green Dot Aviation — 2,9 M vistas — https://youtu.be/9vFTMe0CqBY
+«La desesperación del piloto causó este accidente | Spanair 5022» — Codigo7700 — 1,2 M vistas — https://youtu.be/9totoDNey_s
+«Historias Innecesarias: El Vuelo JK5022» — Historias Innecesarias — 537 k vistas — https://youtu.be/hmcUA4XRwok</t>
         </is>
       </c>
       <c r="E8" s="48" t="inlineStr">
@@ -856,9 +855,9 @@
       </c>
       <c r="D9" s="56" t="inlineStr">
         <is>
-          <t>Ministerio del Interior, detenciones en Ibiza: https://www.interior.gob.es/opencms/en/detail-pages/article/La-Policia-Nacional-detiene-en-Ibiza-a-tres-importantes-miembros-de-la-mafia-calabresa-conocida-como-la-Ndrangheta/
-Última Hora, detenido en Benalmádena: https://www.ultimahora.es/noticias/comunidades/2023/05/04/1930009/detenido-benalmadena-malaga-miembro-ndrangheta-coordinaba-envios-droga-espana-italia.html
-Estilo del canal (vídeos propios): https://youtu.be/dUcXsIlF1E8 · https://youtu.be/Sy6zH00Lr6I</t>
+          <t>«Antonio Pelle, boss di 'ndrangheta - Kings of Crime  CANALE NOVE» — Roberto Saviano Official — 7,0 M vistas — https://youtu.be/3HxyqUDq2pI
+«Mächtig und verschwiegen: So arbeitet die 'Ndrangheta in Deutschland | STRG_F» — STRG_F — 4,0 M vistas — https://youtu.be/YMDmy3LdKGs
+«Breaking the Calabrian Mafia in Italy | Foreign Correspondent» — ABC News In-depth — 3,4 M vistas — https://youtu.be/xZSa4B37sZs</t>
         </is>
       </c>
       <c r="E9" s="56" t="inlineStr">
@@ -893,9 +892,9 @@
       </c>
       <c r="D10" s="60" t="inlineStr">
         <is>
-          <t>Noticias ONU (informe ACNUDH 2023): https://news.un.org/en/node/1140187
-Otras fuentes: UNODC, OCCRP, AP
-Estilo del canal (vídeos propios): https://youtu.be/Sy6zH00Lr6I · https://youtu.be/dUcXsIlF1E8</t>
+          <t>«Inside a Pig Butchering Scam» — Jim Browning — 4,4 M vistas — https://youtu.be/vu-Y1h9rTUs
+«What the Hell Is Happening in Cambodia? | AB Explained» — Asian Boss — 2,2 M vistas — https://youtu.be/n6kbJ9wV5_k
+«Human trafficking victims tortured into scamming innocent people | 60 Minutes Australia» — 60 Minutes Australia — 1,4 M vistas — https://youtu.be/7b7JAX03x2Q</t>
         </is>
       </c>
       <c r="E10" s="60" t="inlineStr">
@@ -930,8 +929,8 @@
       </c>
       <c r="D11" s="44" t="inlineStr">
         <is>
-          <t>Fuentes usadas: Wikipedia (ES/EN), ESDiario 2025, El Debate 2025, Infobae 2023
-Estilo del canal (vídeo propio): https://youtu.be/X22TEmEPZSs</t>
+          <t>«Caso Urquijo: El lugar del crimen» — jm o — 846 k vistas — https://youtu.be/7t5fGz4eVDE
+«EL CASO DE LOS MARQUESES DE URQUIJO · MADRID, 1980 · TINTA ROJA CANAL» — Tinta roja  — 168 k vistas — https://youtu.be/HmS86ch6oA8</t>
         </is>
       </c>
       <c r="E11" s="44" t="inlineStr">
@@ -966,8 +965,8 @@
       </c>
       <c r="D12" s="48" t="inlineStr">
         <is>
-          <t>Fuentes usadas: Wikipedia EN, El Debate 2023 y 2025, Cuatro 2024, COPE 2024, Vozpópuli
-Estilo del canal (vídeo propio): https://youtu.be/X22TEmEPZSs</t>
+          <t>«El desconcertante y durísimo caso del ASESINO DE LA BARAJA contado por Carles Porta de Crims» — The Wild Project — 2,0 M vistas — https://youtu.be/Mx3jIDeHW8k
+«EL PRIMER ASESINO EN SERIE DE ESPAÑA, JOAQUÍN FERRANDIZ - True Crime narrado por Vicente Garrido» — The Wild Project — 3,4 M vistas — https://youtu.be/Sd8wveSzjfI</t>
         </is>
       </c>
       <c r="E12" s="48" t="inlineStr">
@@ -1002,9 +1001,9 @@
       </c>
       <c r="D13" s="56" t="inlineStr">
         <is>
-          <t>Textos: Éxodo 25; 1 Reyes 8; 2 Reyes 25; 2 Macabeos 2; Jeremías 3:16
-Fuentes usadas: Pilgrimaps, Biblical Archaeology Review, Daily Beast
-Estilo del canal (vídeo propio): https://youtu.be/vfMEv2tHywg</t>
+          <t>«EL ARCA DE LA ALIANZA PUEDE HABERSE ENCONTRADO - Arqueólogo ha estado en el templo en el que estaría» — The Wild Project — 1,4 M vistas — https://youtu.be/WimnTTj1Ips
+«Is the Ark of the Covenant REALLY lost?» — hochelaga — 3,3 M vistas — https://youtu.be/_9sTr6n0MFc
+«The Quest To Find The Ark Of The Covenant In Ethiopia | Keepers Of The Lost Ark | Timeline» — Timeline - World History Documentaries — 2,3 M vistas — https://youtu.be/JFxaZ-dkebw</t>
         </is>
       </c>
       <c r="E13" s="56" t="inlineStr">
@@ -1039,9 +1038,8 @@
       </c>
       <c r="D14" s="60" t="inlineStr">
         <is>
-          <t>Biblioteca Digital Leon Levy de los Manuscritos del Mar Muerto (Autoridad de Antigüedades de Israel): https://www.deadseascrolls.org.il
-Fuentes usadas: Jewish Virtual Library, L. Schiffman, Universidad de Groningen 2025
-Estilo del canal (vídeo propio): https://youtu.be/vfMEv2tHywg</t>
+          <t>«Este Es El Descubrimiento Arqueológico Más Importante del Siglo XX» — Historia Incomprendida — 1,8 M vistas — https://youtu.be/LNf4rj4QM5k
+«¿Qué revelan los manuscritos del Mar Muerto? | Julio Trebolle y Florentino García Martínez» — Fundación Juan March — 1,2 M vistas — https://youtu.be/OfCCfAI4nQ4</t>
         </is>
       </c>
       <c r="E14" s="60" t="inlineStr">
@@ -1076,8 +1074,9 @@
       </c>
       <c r="D15" s="44" t="inlineStr">
         <is>
-          <t>Fuentes usadas: World History Encyclopedia, History.com, History Hit, LibreTexts
-Estilo del canal (vídeo propio): https://youtu.be/T4GgahAxokM</t>
+          <t>«What If the Roman Empire NEVER Fell» — The Infographics Show — 951 k vistas — https://youtu.be/se7YNpunwMw
+«What if the Roman Empire Never Fell?» — Whatifalthist — 540 k vistas — https://youtu.be/lisdcxuGSgs
+«¿Y si el IMPERIO ESPAÑOL no hubiera CAÍDO?» — ¿Y si? — 831 k vistas — https://youtu.be/IN6TD1oYbwE</t>
         </is>
       </c>
       <c r="E15" s="44" t="inlineStr">
@@ -1112,8 +1111,8 @@
       </c>
       <c r="D16" s="48" t="inlineStr">
         <is>
-          <t>Universidad Monash (estudio 2024 sobre un posible anillo hace 466 millones de años): https://www.monash.edu/science/news-events/news/2024/earth-may-have-had-a-ring-system-466-million-years-ago
-Estilo del canal (vídeo propio): https://youtu.be/WpwpWOELMJM</t>
+          <t>«¿Qué pasaría si la Tierra tuviera anillos como Saturno?» — Qué pasaría si - What If Español — 2,9 M vistas — https://youtu.be/FK9XRJfxQ5Y
+«What If Earth Had Rings Like Saturn Tomorrow?» — What If — 5,0 M vistas — https://youtu.be/an7FRVPPpW8</t>
         </is>
       </c>
       <c r="E16" s="48" t="inlineStr">

</xml_diff>

<commit_message>
PX-01: página de guiones con enlace por vídeo en la hoja de solicitudes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
@@ -788,14 +788,12 @@
       </c>
       <c r="E7" s="44" t="inlineStr">
         <is>
-          <t>Tono formal pero entretenido, tensión real sin sensacionalismo. Recreaciones 3D realistas del avión, mapas de ruta y diagramas sencillos. Evitar: recrear el impacto, restos o víctimas; fotos de víctimas, supervivientes o tripulantes sin licencia. Pantalla final: vídeo de Helios 522 (https://youtu.be/v3ff8dfP-bs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 01_jager-aviacion_japan-airlines-123.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 1).</t>
+          <t>Tono formal pero entretenido, tensión real sin sensacionalismo. Recreaciones 3D realistas del avión, mapas de ruta y diagramas sencillos. Evitar: recrear el impacto, restos o víctimas; fotos de víctimas, supervivientes o tripulantes sin licencia. Pantalla final: vídeo de Helios 522 (https://youtu.be/v3ff8dfP-bs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F7" s="44" t="inlineStr">
         <is>
-          <t>Guion: 01_jager-aviacion_japan-airlines-123.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 1
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 01: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-01</t>
         </is>
       </c>
     </row>
@@ -825,14 +823,12 @@
       </c>
       <c r="E8" s="48" t="inlineStr">
         <is>
-          <t>Tono formal pero entretenido, explicación técnica clara (flaps, slats, alarma de configuración). Respeto máximo: es un accidente español con familias muy presentes; nada de imágenes del accidente ni de víctimas. Pantalla final: Tenerife 1977 (https://youtu.be/yY81zmnuDEk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 02_jager-aviacion_spanair-jk5022.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 2).</t>
+          <t>Tono formal pero entretenido, explicación técnica clara (flaps, slats, alarma de configuración). Respeto máximo: es un accidente español con familias muy presentes; nada de imágenes del accidente ni de víctimas. Pantalla final: Tenerife 1977 (https://youtu.be/yY81zmnuDEk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F8" s="48" t="inlineStr">
         <is>
-          <t>Guion: 02_jager-aviacion_spanair-jk5022.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 2
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 02: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-02</t>
         </is>
       </c>
     </row>
@@ -862,14 +858,12 @@
       </c>
       <c r="E9" s="56" t="inlineStr">
         <is>
-          <t>Tono informal y burlón contra los criminales; serio en los pasajes de víctimas (Lea Garofalo, Duisburgo). Estética realista desaturada, mapas, organigramas y cifras grandes. Evitar: glorificar, detalles de cómo se oculta la droga, fotos de detenidos sin licencia. Pantalla final: Policía antidroga (https://youtu.be/dUcXsIlF1E8) + botón de suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 03_codigo-mafia_ndrangheta-espana.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 3).</t>
+          <t>Tono informal y burlón contra los criminales; serio en los pasajes de víctimas (Lea Garofalo, Duisburgo). Estética realista desaturada, mapas, organigramas y cifras grandes. Evitar: glorificar, detalles de cómo se oculta la droga, fotos de detenidos sin licencia. Pantalla final: Policía antidroga (https://youtu.be/dUcXsIlF1E8) + botón de suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F9" s="56" t="inlineStr">
         <is>
-          <t>Guion: 03_codigo-mafia_ndrangheta-espana.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 3
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 03: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-03</t>
         </is>
       </c>
     </row>
@@ -899,14 +893,12 @@
       </c>
       <c r="E10" s="60" t="inlineStr">
         <is>
-          <t>Tono informal y burlón contra los jefes de las redes; nunca contra las víctimas (estafados ni trabajadores retenidos). Tono serio en la parte de abusos, sin recrear violencia. Chen Zhi / Prince Group siempre «acusado, no condenado». Sin logotipos de WhatsApp/Telegram ni capturas reales de plataformas. Pantalla final: Telegram (https://youtu.be/Sy6zH00Lr6I) + suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 04_codigo-mafia_complejos-ciberestafa.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 4).</t>
+          <t>Tono informal y burlón contra los jefes de las redes; nunca contra las víctimas (estafados ni trabajadores retenidos). Tono serio en la parte de abusos, sin recrear violencia. Chen Zhi / Prince Group siempre «acusado, no condenado». Sin logotipos de WhatsApp/Telegram ni capturas reales de plataformas. Pantalla final: Telegram (https://youtu.be/Sy6zH00Lr6I) + suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F10" s="60" t="inlineStr">
         <is>
-          <t>Guion: 04_codigo-mafia_complejos-ciberestafa.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 4
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 04: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-04</t>
         </is>
       </c>
     </row>
@@ -935,14 +927,12 @@
       </c>
       <c r="E11" s="44" t="inlineStr">
         <is>
-          <t>Tono sobrio de expediente, sin humor. Solo se presenta como culpable al condenado (Escobedo); el resto, como sospechas, tal como dice el guion. Nunca recrear los disparos ni los cuerpos; portadas de prensa recreadas, no reales. Publicar antes que «El asesino de la baraja» (su pantalla final apunta aquí). Pantalla final: La Viuda Negra de Valencia (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 05_jager-crime_marqueses-urquijo.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 5).</t>
+          <t>Tono sobrio de expediente, sin humor. Solo se presenta como culpable al condenado (Escobedo); el resto, como sospechas, tal como dice el guion. Nunca recrear los disparos ni los cuerpos; portadas de prensa recreadas, no reales. Publicar antes que «El asesino de la baraja» (su pantalla final apunta aquí). Pantalla final: La Viuda Negra de Valencia (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F11" s="44" t="inlineStr">
         <is>
-          <t>Guion: 05_jager-crime_marqueses-urquijo.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 5
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 05: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-05</t>
         </is>
       </c>
     </row>
@@ -971,14 +961,12 @@
       </c>
       <c r="E12" s="48" t="inlineStr">
         <is>
-          <t>Tono sobrio de expediente, sin humor. Respeto a las víctimas: sin recrear los ataques. Alfredo Galán sin foto en primer plano salvo licencia; arma solo en silueta genérica; serie de Netflix sin logotipo. Pantalla final: vídeo de Urquijo (este mismo pedido) o, si aún no está publicado, la Viuda Negra (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 06_jager-crime_asesino-baraja.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 6).</t>
+          <t>Tono sobrio de expediente, sin humor. Respeto a las víctimas: sin recrear los ataques. Alfredo Galán sin foto en primer plano salvo licencia; arma solo en silueta genérica; serie de Netflix sin logotipo. Pantalla final: vídeo de Urquijo (este mismo pedido) o, si aún no está publicado, la Viuda Negra (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F12" s="48" t="inlineStr">
         <is>
-          <t>Guion: 06_jager-crime_asesino-baraja.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 6
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 06: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-06</t>
         </is>
       </c>
     </row>
@@ -1008,14 +996,12 @@
       </c>
       <c r="E13" s="56" t="inlineStr">
         <is>
-          <t>Tono misterioso y envolvente, hablando de tú. Mostrar claras las etiquetas TEXTO / TRADICIÓN / EVIDENCIA. Respeto a creyentes y no creyentes. Sin imágenes de películas (Indiana Jones) ni fotos reales sin licencia. Publicar antes que «Manuscritos del Mar Muerto» (su pantalla final apunta aquí). Pantalla final: Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 07_archivos-sagrados_arca-alianza.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 7).</t>
+          <t>Tono misterioso y envolvente, hablando de tú. Mostrar claras las etiquetas TEXTO / TRADICIÓN / EVIDENCIA. Respeto a creyentes y no creyentes. Sin imágenes de películas (Indiana Jones) ni fotos reales sin licencia. Publicar antes que «Manuscritos del Mar Muerto» (su pantalla final apunta aquí). Pantalla final: Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F13" s="56" t="inlineStr">
         <is>
-          <t>Guion: 07_archivos-sagrados_arca-alianza.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 7
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 07: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-07</t>
         </is>
       </c>
     </row>
@@ -1044,14 +1030,12 @@
       </c>
       <c r="E14" s="60" t="inlineStr">
         <is>
-          <t>Tono misterioso, hablando de tú; etiquetas TEXTO / TRADICIÓN / EVIDENCIA. El anuncio del periódico de 1954, recreado (no la página original sin licencia). Pantalla final: vídeo del Arca (este mismo pedido) o, si aún no está publicado, Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 08_archivos-sagrados_manuscritos-mar-muerto.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 8).</t>
+          <t>Tono misterioso, hablando de tú; etiquetas TEXTO / TRADICIÓN / EVIDENCIA. El anuncio del periódico de 1954, recreado (no la página original sin licencia). Pantalla final: vídeo del Arca (este mismo pedido) o, si aún no está publicado, Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F14" s="60" t="inlineStr">
         <is>
-          <t>Guion: 08_archivos-sagrados_manuscritos-mar-muerto.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 8
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 08: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-08</t>
         </is>
       </c>
     </row>
@@ -1081,14 +1065,12 @@
       </c>
       <c r="E15" s="44" t="inlineStr">
         <is>
-          <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos HISTORIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: Si Colón nunca hubiera llegado a América (https://youtu.be/T4GgahAxokM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 09_jager-explica_si-roma-no-hubiera-caido.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 9).</t>
+          <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos HISTORIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: Si Colón nunca hubiera llegado a América (https://youtu.be/T4GgahAxokM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F15" s="44" t="inlineStr">
         <is>
-          <t>Guion: 09_jager-explica_si-roma-no-hubiera-caido.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 9
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 09: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-09</t>
         </is>
       </c>
     </row>
@@ -1117,14 +1099,12 @@
       </c>
       <c r="E16" s="48" t="inlineStr">
         <is>
-          <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos CIENCIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: El falso vacío (https://youtu.be/WpwpWOELMJM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): 10_jager-explica_si-la-tierra-tuviera-anillos.txt. Descripción de edición bloque a bloque, observaciones y miniatura en el documento del pedido (PX-01.md, vídeo 10).</t>
+          <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos CIENCIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: El falso vacío (https://youtu.be/WpwpWOELMJM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
       <c r="F16" s="48" t="inlineStr">
         <is>
-          <t>Guion: 10_jager-explica_si-la-tierra-tuviera-anillos.txt
-Documento del pedido (edición, observaciones, miniatura): PX-01.md, vídeo 10
-[Pegar aquí el enlace de Drive con acceso concedido]</t>
+          <t>Guion 10: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
PX-01: enlaces clicables por guion; la página muestra solo el guion enlazado
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
@@ -13,7 +13,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <name val="Carlito"/>
       <sz val="11"/>
@@ -72,6 +72,12 @@
       <name val="Carlito"/>
       <b val="1"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Carlito"/>
+      <color rgb="FF1F5FAD"/>
+      <sz val="11"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="16">
@@ -165,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -401,6 +407,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -791,9 +809,9 @@
           <t>Tono formal pero entretenido, tensión real sin sensacionalismo. Recreaciones 3D realistas del avión, mapas de ruta y diagramas sencillos. Evitar: recrear el impacto, restos o víctimas; fotos de víctimas, supervivientes o tripulantes sin licencia. Pantalla final: vídeo de Helios 522 (https://youtu.be/v3ff8dfP-bs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F7" s="44" t="inlineStr">
-        <is>
-          <t>Guion 01: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-01</t>
+      <c r="F7" s="104" t="inlineStr">
+        <is>
+          <t>Abrir guion 01</t>
         </is>
       </c>
     </row>
@@ -826,9 +844,9 @@
           <t>Tono formal pero entretenido, explicación técnica clara (flaps, slats, alarma de configuración). Respeto máximo: es un accidente español con familias muy presentes; nada de imágenes del accidente ni de víctimas. Pantalla final: Tenerife 1977 (https://youtu.be/yY81zmnuDEk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F8" s="48" t="inlineStr">
-        <is>
-          <t>Guion 02: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-02</t>
+      <c r="F8" s="105" t="inlineStr">
+        <is>
+          <t>Abrir guion 02</t>
         </is>
       </c>
     </row>
@@ -861,9 +879,9 @@
           <t>Tono informal y burlón contra los criminales; serio en los pasajes de víctimas (Lea Garofalo, Duisburgo). Estética realista desaturada, mapas, organigramas y cifras grandes. Evitar: glorificar, detalles de cómo se oculta la droga, fotos de detenidos sin licencia. Pantalla final: Policía antidroga (https://youtu.be/dUcXsIlF1E8) + botón de suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F9" s="56" t="inlineStr">
-        <is>
-          <t>Guion 03: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-03</t>
+      <c r="F9" s="106" t="inlineStr">
+        <is>
+          <t>Abrir guion 03</t>
         </is>
       </c>
     </row>
@@ -896,9 +914,9 @@
           <t>Tono informal y burlón contra los jefes de las redes; nunca contra las víctimas (estafados ni trabajadores retenidos). Tono serio en la parte de abusos, sin recrear violencia. Chen Zhi / Prince Group siempre «acusado, no condenado». Sin logotipos de WhatsApp/Telegram ni capturas reales de plataformas. Pantalla final: Telegram (https://youtu.be/Sy6zH00Lr6I) + suscripción. Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F10" s="60" t="inlineStr">
-        <is>
-          <t>Guion 04: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-04</t>
+      <c r="F10" s="107" t="inlineStr">
+        <is>
+          <t>Abrir guion 04</t>
         </is>
       </c>
     </row>
@@ -930,9 +948,9 @@
           <t>Tono sobrio de expediente, sin humor. Solo se presenta como culpable al condenado (Escobedo); el resto, como sospechas, tal como dice el guion. Nunca recrear los disparos ni los cuerpos; portadas de prensa recreadas, no reales. Publicar antes que «El asesino de la baraja» (su pantalla final apunta aquí). Pantalla final: La Viuda Negra de Valencia (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F11" s="44" t="inlineStr">
-        <is>
-          <t>Guion 05: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-05</t>
+      <c r="F11" s="104" t="inlineStr">
+        <is>
+          <t>Abrir guion 05</t>
         </is>
       </c>
     </row>
@@ -964,9 +982,9 @@
           <t>Tono sobrio de expediente, sin humor. Respeto a las víctimas: sin recrear los ataques. Alfredo Galán sin foto en primer plano salvo licencia; arma solo en silueta genérica; serie de Netflix sin logotipo. Pantalla final: vídeo de Urquijo (este mismo pedido) o, si aún no está publicado, la Viuda Negra (https://youtu.be/X22TEmEPZSs). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F12" s="48" t="inlineStr">
-        <is>
-          <t>Guion 06: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-06</t>
+      <c r="F12" s="105" t="inlineStr">
+        <is>
+          <t>Abrir guion 06</t>
         </is>
       </c>
     </row>
@@ -999,9 +1017,9 @@
           <t>Tono misterioso y envolvente, hablando de tú. Mostrar claras las etiquetas TEXTO / TRADICIÓN / EVIDENCIA. Respeto a creyentes y no creyentes. Sin imágenes de películas (Indiana Jones) ni fotos reales sin licencia. Publicar antes que «Manuscritos del Mar Muerto» (su pantalla final apunta aquí). Pantalla final: Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F13" s="56" t="inlineStr">
-        <is>
-          <t>Guion 07: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-07</t>
+      <c r="F13" s="106" t="inlineStr">
+        <is>
+          <t>Abrir guion 07</t>
         </is>
       </c>
     </row>
@@ -1033,9 +1051,9 @@
           <t>Tono misterioso, hablando de tú; etiquetas TEXTO / TRADICIÓN / EVIDENCIA. El anuncio del periódico de 1954, recreado (no la página original sin licencia). Pantalla final: vídeo del Arca (este mismo pedido) o, si aún no está publicado, Los gigantes de la Biblia (https://youtu.be/fd9JRC_2AXk). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F14" s="60" t="inlineStr">
-        <is>
-          <t>Guion 08: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-08</t>
+      <c r="F14" s="107" t="inlineStr">
+        <is>
+          <t>Abrir guion 08</t>
         </is>
       </c>
     </row>
@@ -1068,9 +1086,9 @@
           <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos HISTORIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: Si Colón nunca hubiera llegado a América (https://youtu.be/T4GgahAxokM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F15" s="44" t="inlineStr">
-        <is>
-          <t>Guion 09: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-09</t>
+      <c r="F15" s="104" t="inlineStr">
+        <is>
+          <t>Abrir guion 09</t>
         </is>
       </c>
     </row>
@@ -1102,9 +1120,9 @@
           <t>Tono divertido y enérgico, comparaciones absurdas. Vídeo normal: imágenes reales o de archivo y recreaciones; sin animación, sin personaje y sin presentador. Sellos CIENCIA (dato real) e IMAGINANDO (especulación) bien visibles. Pantalla final: El falso vacío (https://youtu.be/WpwpWOELMJM). Guion de unas 3.800 palabras (≈ 20-25 min según la velocidad de la voz). Guion completo escrito por nosotros (no hace falta redactarlo): enlace en «Archivos Necesarios».</t>
         </is>
       </c>
-      <c r="F16" s="48" t="inlineStr">
-        <is>
-          <t>Guion 10: https://claude.ai/artifact/3BNFj9F2s71kMAAAGwx81t#guion-10</t>
+      <c r="F16" s="105" t="inlineStr">
+        <is>
+          <t>Abrir guion 10</t>
         </is>
       </c>
     </row>
@@ -1212,6 +1230,18 @@
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="A22:B22"/>
   </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId10"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
PX-01: enlaces de Drive visibles en hoja y documento del pedido
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013kFn69JUwjpJLGjYQm3cxD
</commit_message>
<xml_diff>
--- a/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
+++ b/ESTUDIO/PEDIDOS_PIXELIDO/solicitudes_PX-01_10_videos.xlsx
@@ -811,7 +811,7 @@
       </c>
       <c r="F7" s="104" t="inlineStr">
         <is>
-          <t>Abrir guion 01</t>
+          <t>Guion 01: https://docs.google.com/document/d/1XAsgsvRm8LlnGcCXyFNwkVd_xGNvJmDzyhLUeD8B1ag/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
       </c>
       <c r="F8" s="105" t="inlineStr">
         <is>
-          <t>Abrir guion 02</t>
+          <t>Guion 02: https://docs.google.com/document/d/1FfI-oQLIrUbG4HLaaXq_74eSuRWBFeEtDGJu8rzvdBU/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="F9" s="106" t="inlineStr">
         <is>
-          <t>Abrir guion 03</t>
+          <t>Guion 03: https://docs.google.com/document/d/1ST3Gso-NKBWovm64_yXa8k2QAmZLPLuR_3VX6rP6Fyc/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="F10" s="107" t="inlineStr">
         <is>
-          <t>Abrir guion 04</t>
+          <t>Guion 04: https://docs.google.com/document/d/1zrhWZ7wj7AdboTMtXfSkoYYGNW22cHB8Ct6TEkLec4U/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -950,7 +950,7 @@
       </c>
       <c r="F11" s="104" t="inlineStr">
         <is>
-          <t>Abrir guion 05</t>
+          <t>Guion 05: https://docs.google.com/document/d/1_7jDQm4SSNQTpeKOc_eKkh9BZ-D6iEJta2gpNlTfcFI/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -984,7 +984,7 @@
       </c>
       <c r="F12" s="105" t="inlineStr">
         <is>
-          <t>Abrir guion 06</t>
+          <t>Guion 06: https://docs.google.com/document/d/1YyiHILOdcJ6L80h3h3hf-QI9jNYjAyM-clkUINZhsaI/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="F13" s="106" t="inlineStr">
         <is>
-          <t>Abrir guion 07</t>
+          <t>Guion 07: https://docs.google.com/document/d/1BOOR8JSo80ZmkLFuoWeqoB00HLK9GrbZlVmkWm3cACA/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -1053,7 +1053,7 @@
       </c>
       <c r="F14" s="107" t="inlineStr">
         <is>
-          <t>Abrir guion 08</t>
+          <t>Guion 08: https://docs.google.com/document/d/1frA1g8llaLuK1w512pc4oFtyPkQa-eTqLszkEREvLUQ/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
       </c>
       <c r="F15" s="104" t="inlineStr">
         <is>
-          <t>Abrir guion 09</t>
+          <t>Guion 09: https://docs.google.com/document/d/1k6pcxbByIhiqZSe56gCv4TaK5bjqZXcT0FHSbxwnors/edit?usp=sharing</t>
         </is>
       </c>
     </row>
@@ -1122,7 +1122,7 @@
       </c>
       <c r="F16" s="105" t="inlineStr">
         <is>
-          <t>Abrir guion 10</t>
+          <t>Guion 10: https://docs.google.com/document/d/1aT8tTbo-Gaw8-U8rektsywB_c6wDRaAw04uyeWTI-nE/edit?usp=sharing</t>
         </is>
       </c>
     </row>

</xml_diff>